<commit_message>
more error checking scripts
</commit_message>
<xml_diff>
--- a/Excel/3_1_Enteric_Feedlot_WIP_v02.xlsx
+++ b/Excel/3_1_Enteric_Feedlot_WIP_v02.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F22FEC59-8416-4BD5-B021-0F8403D6FB99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A70D020C-FA80-4211-8B34-9B0A2B3369A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="37170" windowHeight="19920" activeTab="3" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="28800" windowHeight="15345" activeTab="3" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -438,6 +438,7 @@
     <definedName name="Table_D_j">'3.1.1.1-2 Enteric Methane'!$D$54:$F$55</definedName>
     <definedName name="Table_N_j">'3.1.1.1-2 Enteric Methane'!$D$59:$F$60</definedName>
     <definedName name="VEERG_3_1_1_1__1_TotalAnnualMethaneFromEntericFermentation_Result">'3.1.1.1-2 Enteric Methane'!$E$67</definedName>
+    <definedName name="VEERG_3_1_1_1__1_TotalAnnualMethaneFromEntericFermentation_Result_Method2">'3.1.1.1-2 Enteric Methane'!$N$67</definedName>
     <definedName name="X_Table_Feedlot_HerdMovement">'Input - Feedlot'!$D$7:$G$9</definedName>
     <definedName name="X_Table_Feedlot_Intake_Method1">'Input - Feedlot'!$D$13:$G$16</definedName>
     <definedName name="X_Table_Feedlot_Intake_Method2">'Input - Feedlot'!$D$18:$G$21</definedName>
@@ -2654,32 +2655,6 @@
   <dxfs count="77">
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFB2D498"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -3565,6 +3540,32 @@
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFB2D498"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -6174,34 +6175,34 @@
     <tableColumn id="1" xr3:uid="{3885FE93-299E-44EB-B503-99C305BD6F41}" name="Treatment stage T">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{D0E12F95-AC29-47D0-913A-0A0B02931616}" name="MMS m" dataDxfId="27" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{D0E12F95-AC29-47D0-913A-0A0B02931616}" name="MMS m" dataDxfId="64" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{E17BE7AB-8FAD-4B5C-9F86-E70E6A00B9B1}" name="NSW" dataDxfId="26" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{E17BE7AB-8FAD-4B5C-9F86-E70E6A00B9B1}" name="NSW" dataDxfId="63" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{D4C6F922-2719-4479-B7CC-26C5286F73ED}" name="ACT" dataDxfId="25" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{D4C6F922-2719-4479-B7CC-26C5286F73ED}" name="ACT" dataDxfId="62" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{5034DCA1-F046-43BC-A94F-832832E6D634}" name="QLD" dataDxfId="24" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{5034DCA1-F046-43BC-A94F-832832E6D634}" name="QLD" dataDxfId="61" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{186521AB-DFC2-4E3B-A674-A5382DCC5ACD}" name="NT" dataDxfId="23" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{186521AB-DFC2-4E3B-A674-A5382DCC5ACD}" name="NT" dataDxfId="60" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{95F9E197-F85F-424A-B68D-774604116729}" name="SA" dataDxfId="22" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{95F9E197-F85F-424A-B68D-774604116729}" name="SA" dataDxfId="59" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{A6DDF652-660B-4C41-982D-FECC3B1142AF}" name="VIC" dataDxfId="21" dataCellStyle="Content normal">
+    <tableColumn id="8" xr3:uid="{A6DDF652-660B-4C41-982D-FECC3B1142AF}" name="VIC" dataDxfId="58" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{5163E1D2-D984-4DBA-95A9-1667F628B2D9}" name="WA" dataDxfId="20" dataCellStyle="Content normal">
+    <tableColumn id="9" xr3:uid="{5163E1D2-D984-4DBA-95A9-1667F628B2D9}" name="WA" dataDxfId="57" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{A0E67108-978C-4849-A310-69F8E4739C6D}" name="TAS" dataDxfId="19" dataCellStyle="Content normal">
+    <tableColumn id="10" xr3:uid="{A0E67108-978C-4849-A310-69F8E4739C6D}" name="TAS" dataDxfId="56" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{27E929DD-0554-43B8-A58C-34B0A39F2EBA}" name="NIR definition" dataDxfId="18" dataCellStyle="Content normal">
+    <tableColumn id="11" xr3:uid="{27E929DD-0554-43B8-A58C-34B0A39F2EBA}" name="NIR definition" dataDxfId="55" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6317,49 +6318,49 @@
     <tableColumn id="1" xr3:uid="{712516A0-1F9E-4023-BA82-6672681A870F}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{11C0CC10-B6D1-4F1B-AF67-63540D3C6573}" name="MAT" totalsRowDxfId="64" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{11C0CC10-B6D1-4F1B-AF67-63540D3C6573}" name="MAT" totalsRowDxfId="36" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B2E86635-9B5F-4851-B090-DE2ACAEDF447}" name="MAP" totalsRowDxfId="63" totalsRowCellStyle="Content bold">
+    <tableColumn id="3" xr3:uid="{B2E86635-9B5F-4851-B090-DE2ACAEDF447}" name="MAP" totalsRowDxfId="35" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{7F73CA39-E92F-4A10-8511-3C929BFEDAA2}" name="Frost days per year" totalsRowDxfId="62" totalsRowCellStyle="Content bold">
+    <tableColumn id="4" xr3:uid="{7F73CA39-E92F-4A10-8511-3C929BFEDAA2}" name="Frost days per year" totalsRowDxfId="34" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{1B756309-A904-4B03-89BB-F0E9CFE961A2}" name="Elevation" totalsRowDxfId="61" totalsRowCellStyle="Content bold">
+    <tableColumn id="5" xr3:uid="{1B756309-A904-4B03-89BB-F0E9CFE961A2}" name="Elevation" totalsRowDxfId="33" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{ECCF8CE7-918B-424A-8D0B-FE1A50768C61}" name="MAP:PET" totalsRowDxfId="60" totalsRowCellStyle="Content bold">
+    <tableColumn id="6" xr3:uid="{ECCF8CE7-918B-424A-8D0B-FE1A50768C61}" name="MAP:PET" totalsRowDxfId="32" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{9F97F8D6-CC77-43B2-A9DF-16FA34A0821C}" name="Min temp" totalsRowDxfId="59" totalsRowCellStyle="Content bold">
+    <tableColumn id="7" xr3:uid="{9F97F8D6-CC77-43B2-A9DF-16FA34A0821C}" name="Min temp" totalsRowDxfId="31" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{F368831A-6ABD-4702-AD6C-40392EBDF102}" name="Max temp" totalsRowDxfId="58" totalsRowCellStyle="Content bold">
+    <tableColumn id="8" xr3:uid="{F368831A-6ABD-4702-AD6C-40392EBDF102}" name="Max temp" totalsRowDxfId="30" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{394284B4-1932-4CF9-87A0-10AC0C355803}" name="Min rainfall" totalsRowDxfId="57" totalsRowCellStyle="Content bold">
+    <tableColumn id="9" xr3:uid="{394284B4-1932-4CF9-87A0-10AC0C355803}" name="Min rainfall" totalsRowDxfId="29" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{39B4AC69-0BE8-4809-88BD-3D9C3366C801}" name="Max rainfall" totalsRowDxfId="56" totalsRowCellStyle="Content bold">
+    <tableColumn id="10" xr3:uid="{39B4AC69-0BE8-4809-88BD-3D9C3366C801}" name="Max rainfall" totalsRowDxfId="28" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{C52624FB-1991-4D08-BF77-8867175351D7}" name="Min frost days" totalsRowDxfId="55" totalsRowCellStyle="Content bold">
+    <tableColumn id="11" xr3:uid="{C52624FB-1991-4D08-BF77-8867175351D7}" name="Min frost days" totalsRowDxfId="27" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{4AF5B2C1-2CB6-41E8-98B7-F05A02BE5CCF}" name="Max frost days" totalsRowDxfId="54" totalsRowCellStyle="Content bold">
+    <tableColumn id="15" xr3:uid="{4AF5B2C1-2CB6-41E8-98B7-F05A02BE5CCF}" name="Max frost days" totalsRowDxfId="26" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{DC14DCAE-993A-4A49-B055-B24393671D48}" name="Min elevation" totalsRowDxfId="53" totalsRowCellStyle="Content bold">
+    <tableColumn id="12" xr3:uid="{DC14DCAE-993A-4A49-B055-B24393671D48}" name="Min elevation" totalsRowDxfId="25" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{9456662F-6E71-4AE4-BED7-B34F70B718EF}" name="Max elevation" totalsRowDxfId="52" totalsRowCellStyle="Content bold">
+    <tableColumn id="16" xr3:uid="{9456662F-6E71-4AE4-BED7-B34F70B718EF}" name="Max elevation" totalsRowDxfId="24" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{43296FE0-60C3-4ECC-B983-CA2EC824388C}" name="Min MAP:PET" totalsRowDxfId="51" totalsRowCellStyle="Content bold">
+    <tableColumn id="13" xr3:uid="{43296FE0-60C3-4ECC-B983-CA2EC824388C}" name="Min MAP:PET" totalsRowDxfId="23" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{E271A63E-F2F9-411F-9BBD-348C53F4E7FA}" name="Max MAP:PET" totalsRowDxfId="50" totalsRowCellStyle="Content bold">
+    <tableColumn id="17" xr3:uid="{E271A63E-F2F9-411F-9BBD-348C53F4E7FA}" name="Max MAP:PET" totalsRowDxfId="22" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6377,7 +6378,7 @@
     <tableColumn id="1" xr3:uid="{C157AB0B-7B8C-47CD-9FE8-5C545E96772B}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{E4F74487-53B1-43B5-B614-8DAD9E2DFFE5}" name="Wet or Dry Zone" totalsRowDxfId="49" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{E4F74487-53B1-43B5-B614-8DAD9E2DFFE5}" name="Wet or Dry Zone" totalsRowDxfId="21" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6481,7 +6482,7 @@
   </autoFilter>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{F2B173A3-CADE-4DCA-988D-39EE2392D8DB}" name="MMS"/>
-    <tableColumn id="2" xr3:uid="{67006656-167A-4452-9820-88D798B88ADD}" name="Symbol and MMS" dataDxfId="17" dataCellStyle="Content normal"/>
+    <tableColumn id="2" xr3:uid="{67006656-167A-4452-9820-88D798B88ADD}" name="Symbol and MMS" dataDxfId="54" dataCellStyle="Content normal"/>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6497,7 +6498,7 @@
     <tableColumn id="1" xr3:uid="{E03AF6FD-C2DC-4E2A-8DD2-9D01C3922F68}" name="Is in leaching zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{5FE7D2C0-93B2-4CFA-8E49-86D22018F701}" name="FracWET" dataDxfId="48">
+    <tableColumn id="2" xr3:uid="{5FE7D2C0-93B2-4CFA-8E49-86D22018F701}" name="FracWET" dataDxfId="20">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6545,7 +6546,7 @@
     <tableColumn id="1" xr3:uid="{350E7C3F-23B3-447B-B4C4-6060BF022EA9}" name="Irrigation type i">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{AAFBF774-1644-4FD1-A124-9B504EDFABE4}" name="FracWET" dataDxfId="47" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{AAFBF774-1644-4FD1-A124-9B504EDFABE4}" name="FracWET" dataDxfId="19" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6563,7 +6564,7 @@
     <tableColumn id="1" xr3:uid="{F53737D0-55CF-4CE4-A2DA-5E64EC681B30}" name="Climate zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{FDEB6DD4-2D71-459B-9A7D-91F401E4C50D}" name="EFPRP" dataDxfId="46" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{FDEB6DD4-2D71-459B-9A7D-91F401E4C50D}" name="EFPRP" dataDxfId="18" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6581,7 +6582,7 @@
     <tableColumn id="1" xr3:uid="{5ACE1312-EFBD-47E7-BAE6-CD1DFB5C1149}" name="Month">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{55926360-A3BF-4F7D-930E-33008C7948DC}" name="Season" dataDxfId="45" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{55926360-A3BF-4F7D-930E-33008C7948DC}" name="Season" dataDxfId="17" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6613,49 +6614,49 @@
     <tableColumn id="1" xr3:uid="{34A8EA66-F024-45E8-B03E-791B841E9749}" name="Temperature zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{B4BFB9E6-B3AE-4AE0-8FC9-A3A15770F2A3}" name="MAT (ºC)" dataDxfId="44" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{B4BFB9E6-B3AE-4AE0-8FC9-A3A15770F2A3}" name="MAT (ºC)" dataDxfId="16" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{1E9D6328-E0CD-4C53-90C0-0E060E861710}" name="Anaerobic lagoon" dataDxfId="43" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{1E9D6328-E0CD-4C53-90C0-0E060E861710}" name="Anaerobic lagoon" dataDxfId="15" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{7E542609-0309-4456-863B-5E7A42AE24FC}" name="Digester / covered lagoons" dataDxfId="42" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{7E542609-0309-4456-863B-5E7A42AE24FC}" name="Digester / covered lagoons" dataDxfId="14" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{6915A606-992F-4E57-AF1B-AD9F7C399E5E}" name="Liquid systems" dataDxfId="41" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{6915A606-992F-4E57-AF1B-AD9F7C399E5E}" name="Liquid systems" dataDxfId="13" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{506F7060-E7A1-4B7A-B0E1-78E30D0BEDED}" name="Daily spread" dataDxfId="40" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{506F7060-E7A1-4B7A-B0E1-78E30D0BEDED}" name="Daily spread" dataDxfId="12" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{0A00F34D-939F-4296-95CC-077DD279A797}" name="Composting (passive windrow)" dataDxfId="39" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{0A00F34D-939F-4296-95CC-077DD279A797}" name="Composting (passive windrow)" dataDxfId="11" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{230EBB79-6A17-4516-80B6-F375FF9669A9}" name="Solid storage" dataDxfId="38" dataCellStyle="Content normal">
+    <tableColumn id="8" xr3:uid="{230EBB79-6A17-4516-80B6-F375FF9669A9}" name="Solid storage" dataDxfId="10" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{85559CD2-6C4D-4F6D-AFDF-9A0890886D97}" name="Pit storage" dataDxfId="37" dataCellStyle="Content normal">
+    <tableColumn id="9" xr3:uid="{85559CD2-6C4D-4F6D-AFDF-9A0890886D97}" name="Pit storage" dataDxfId="9" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{8D428E8C-5F0E-4324-A4B8-393A0103893A}" name="Deep litter" dataDxfId="36" dataCellStyle="Content normal">
+    <tableColumn id="10" xr3:uid="{8D428E8C-5F0E-4324-A4B8-393A0103893A}" name="Deep litter" dataDxfId="8" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{7B3894FD-B1DE-49E3-93E3-9C2D5D5FEFD6}" name="Poultry manure with bedding" dataDxfId="35" dataCellStyle="Content normal">
+    <tableColumn id="11" xr3:uid="{7B3894FD-B1DE-49E3-93E3-9C2D5D5FEFD6}" name="Poultry manure with bedding" dataDxfId="7" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{BB24A1FF-05D1-44A8-885D-770FEC703393}" name="Poultry manure without bedding" dataDxfId="34" dataCellStyle="Content normal">
+    <tableColumn id="12" xr3:uid="{BB24A1FF-05D1-44A8-885D-770FEC703393}" name="Poultry manure without bedding" dataDxfId="6" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{732C2DE9-2AD0-427C-A104-694DE52E31E9}" name="Direct processing" dataDxfId="33" dataCellStyle="Content normal">
+    <tableColumn id="13" xr3:uid="{732C2DE9-2AD0-427C-A104-694DE52E31E9}" name="Direct processing" dataDxfId="5" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{7CA673A4-7283-4EE6-A8B7-7FA16B4D8FC2}" name="Direct application" dataDxfId="32" dataCellStyle="Content normal">
+    <tableColumn id="14" xr3:uid="{7CA673A4-7283-4EE6-A8B7-7FA16B4D8FC2}" name="Direct application" dataDxfId="4" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{A901BEDD-817D-4DC0-8C93-4FA88EFB5BB0}" name="Pasture range and paddock" dataDxfId="31" dataCellStyle="Content normal">
+    <tableColumn id="15" xr3:uid="{A901BEDD-817D-4DC0-8C93-4FA88EFB5BB0}" name="Pasture range and paddock" dataDxfId="3" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{DB14FD26-FA63-40B5-9A79-1EB0E579EFE3}" name="MAT raw" dataDxfId="30" dataCellStyle="Content normal">
+    <tableColumn id="16" xr3:uid="{DB14FD26-FA63-40B5-9A79-1EB0E579EFE3}" name="MAT raw" dataDxfId="2" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6673,7 +6674,7 @@
     <tableColumn id="1" xr3:uid="{C10B0DCC-AB7B-472C-AFA2-D9FBA01FEEFC}" name="Climate Zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{6A330EA4-D04D-4DD5-8483-059B774FB8A7}" name="EFNi &amp; EFN2Oi" dataDxfId="29" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{6A330EA4-D04D-4DD5-8483-059B774FB8A7}" name="EFNi &amp; EFN2Oi" dataDxfId="1" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6689,7 +6690,7 @@
     <filterColumn colId="2" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="3">
-    <tableColumn id="2" xr3:uid="{F4085F84-B7D6-4E41-8C32-36C2B6908D02}" name="Description" dataDxfId="28" dataCellStyle="Content normal"/>
+    <tableColumn id="2" xr3:uid="{F4085F84-B7D6-4E41-8C32-36C2B6908D02}" name="Description" dataDxfId="0" dataCellStyle="Content normal"/>
     <tableColumn id="1" xr3:uid="{C208DBA4-4CA6-4556-839E-BC861134E788}" name="ID"/>
     <tableColumn id="3" xr3:uid="{E813DE45-E616-4D89-AB2F-7A47CC57EA50}" name="Score"/>
   </tableColumns>
@@ -6744,22 +6745,22 @@
     <tableColumn id="1" xr3:uid="{FDCB848C-205F-48EA-BACF-F54BCD324E05}" name="Feedlot type">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{3306F917-B06C-4CC9-B1B1-D97D858E6DAA}" name="Nutrient analysis" dataDxfId="16" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{3306F917-B06C-4CC9-B1B1-D97D858E6DAA}" name="Nutrient analysis" dataDxfId="53" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{F162F7C2-B0FA-499A-BD58-855C4DF97FA8}" name="Unit" dataDxfId="15" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{F162F7C2-B0FA-499A-BD58-855C4DF97FA8}" name="Unit" dataDxfId="52" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{D395A9F5-9A85-4032-A7C1-EC470516DD87}" name="2010-2014" dataDxfId="14" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{D395A9F5-9A85-4032-A7C1-EC470516DD87}" name="2010-2014" dataDxfId="51" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{B149E561-7044-4839-B850-C751ABC364C9}" name="2015-2019" dataDxfId="13" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{B149E561-7044-4839-B850-C751ABC364C9}" name="2015-2019" dataDxfId="50" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{ECEB8E53-4880-43AE-9D36-F969D05BCB18}" name="2020-2023" dataDxfId="12" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{ECEB8E53-4880-43AE-9D36-F969D05BCB18}" name="2020-2023" dataDxfId="49" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{3B7FAEA4-08D7-48B2-9062-7D93639222CC}" name="2020-2023 Converted to fraction" dataDxfId="11" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{3B7FAEA4-08D7-48B2-9062-7D93639222CC}" name="2020-2023 Converted to fraction" dataDxfId="48" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6820,22 +6821,22 @@
     <tableColumn id="1" xr3:uid="{96F6B4E3-E1EE-445F-9BCE-628B89FC3727}" name="Feedlot type">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{6B651FD0-BCF6-4081-8A93-6B21A1D6CA99}" name="Characteristic" dataDxfId="10" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{6B651FD0-BCF6-4081-8A93-6B21A1D6CA99}" name="Characteristic" dataDxfId="47" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{3F266A2B-76EA-4E95-B049-75B8E4AB351F}" name="Unit" dataDxfId="9" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{3F266A2B-76EA-4E95-B049-75B8E4AB351F}" name="Unit" dataDxfId="46" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{15472767-3F72-4A65-88AC-C3242A8E1662}" name="2005-2009" dataDxfId="8" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{15472767-3F72-4A65-88AC-C3242A8E1662}" name="2005-2009" dataDxfId="45" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{5F74A8B9-7EFB-4457-8ADA-5E1ABA9DA889}" name="2010-2014" dataDxfId="7" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{5F74A8B9-7EFB-4457-8ADA-5E1ABA9DA889}" name="2010-2014" dataDxfId="44" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{E54F2812-2E8B-41EB-98A8-46890B5B4E13}" name="2015-2019" dataDxfId="6" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{E54F2812-2E8B-41EB-98A8-46890B5B4E13}" name="2015-2019" dataDxfId="43" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{88EEE0E3-F5D0-41DF-80EF-59472377C29A}" name="2020-2023" dataDxfId="5" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{88EEE0E3-F5D0-41DF-80EF-59472377C29A}" name="2020-2023" dataDxfId="42" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6853,7 +6854,7 @@
     <tableColumn id="1" xr3:uid="{9D472457-4D8B-44ED-9567-B889D058C2F1}" name="Feedlot type">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DurationOfStay_Data(), Table_SourceData_Feedlot_LengthOfStay[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{DA3DA009-634B-4C70-926B-C8FB255EB4DC}" name="Length of stay" dataDxfId="4" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{DA3DA009-634B-4C70-926B-C8FB255EB4DC}" name="Length of stay" dataDxfId="41" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DurationOfStay_Data(), Table_SourceData_Feedlot_LengthOfStay[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6873,13 +6874,13 @@
     <tableColumn id="1" xr3:uid="{C80C08D8-3F48-4E18-98E3-9B53ACB6C6D9}" name="Treatment stage T">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_NitrousOxideEFs_Data(), Table_SourceData_Feedlot_NO2EFs[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{2BCD8589-5CB8-4ED1-AF2B-2866CEF779A8}" name="MMS m" dataDxfId="3" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{2BCD8589-5CB8-4ED1-AF2B-2866CEF779A8}" name="MMS m" dataDxfId="40" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_NitrousOxideEFs_Data(), Table_SourceData_Feedlot_NO2EFs[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{51E876CD-83B6-49C8-85DD-E2F427A3DCD0}" name="EF mT" dataDxfId="2" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{51E876CD-83B6-49C8-85DD-E2F427A3DCD0}" name="EF mT" dataDxfId="39" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_NitrousOxideEFs_Data(), Table_SourceData_Feedlot_NO2EFs[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{BEDEE6BB-8013-495A-8D74-2C8D37558C98}" name="NIR definition" dataDxfId="1" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{BEDEE6BB-8013-495A-8D74-2C8D37558C98}" name="NIR definition" dataDxfId="38" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_NitrousOxideEFs_Data(), Table_SourceData_Feedlot_NO2EFs[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6888,7 +6889,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{100A8309-C0D3-4638-A47B-72840A042D9A}" name="Table_SourceData_Feedlot_FracGASMmT" displayName="Table_SourceData_Feedlot_FracGASMmT" ref="D112:G117" totalsRowShown="0" headerRowDxfId="0" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{100A8309-C0D3-4638-A47B-72840A042D9A}" name="Table_SourceData_Feedlot_FracGASMmT" displayName="Table_SourceData_Feedlot_FracGASMmT" ref="D112:G117" totalsRowShown="0" headerRowDxfId="37" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
   <autoFilter ref="D112:G117" xr:uid="{100A8309-C0D3-4638-A47B-72840A042D9A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -12935,7 +12936,7 @@
         <v>35.420230000000004</v>
       </c>
       <c r="F7" s="94">
-        <f ca="1">'3.1.1.1-2 Enteric Methane'!N67</f>
+        <f ca="1">VEERG_3_1_1_1__1_TotalAnnualMethaneFromEntericFermentation_Result_Method2</f>
         <v>35.420230000000004</v>
       </c>
       <c r="G7" s="50" t="str">

</xml_diff>